<commit_message>
Update: Fixed Description Text bug
</commit_message>
<xml_diff>
--- a/APPT/data/input/packing_plan.xlsx
+++ b/APPT/data/input/packing_plan.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pratyush\Desktop\ARX\ARX-SFA Projects\P&amp;G\PG-AutoProdTool\APPT\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4ED5D6B-D224-45D9-A158-10CC1A3B7589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3478F0F6-EECD-43E0-8660-A6DBE1FD0A10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14310" yWindow="0" windowWidth="14580" windowHeight="17370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Production Schedule Data Transc" sheetId="1" r:id="rId1"/>
+    <sheet name="Production Schedule Data Tr (2)" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="62">
   <si>
     <t>Plant</t>
   </si>
@@ -206,18 +206,6 @@
   </si>
   <si>
     <t>PNTN COND 200MLX 24 HS HF</t>
-  </si>
-  <si>
-    <t>GCAS</t>
-  </si>
-  <si>
-    <t>System</t>
-  </si>
-  <si>
-    <t>6T</t>
-  </si>
-  <si>
-    <t>12T</t>
   </si>
 </sst>
 </file>
@@ -483,30 +471,30 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:T36"/>
+  <dimension ref="A1:R36"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.7265625" customWidth="1"/>
-    <col min="2" max="2" width="12.6328125" customWidth="1"/>
-    <col min="3" max="3" width="7.90625" customWidth="1"/>
-    <col min="4" max="4" width="9.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.36328125" customWidth="1"/>
-    <col min="6" max="6" width="37.08984375" customWidth="1"/>
-    <col min="7" max="9" width="10.453125" customWidth="1"/>
-    <col min="10" max="10" width="9.36328125" customWidth="1"/>
-    <col min="11" max="11" width="8.6328125" customWidth="1"/>
-    <col min="12" max="12" width="9.36328125" customWidth="1"/>
-    <col min="13" max="13" width="8.08984375" customWidth="1"/>
-    <col min="14" max="14" width="13.7265625" customWidth="1"/>
-    <col min="15" max="15" width="11.08984375" customWidth="1"/>
-    <col min="16" max="16" width="11.7265625" customWidth="1"/>
-    <col min="17" max="17" width="12.7265625" customWidth="1"/>
-    <col min="18" max="18" width="28.6328125" customWidth="1"/>
-    <col min="19" max="19" width="12.7265625" customWidth="1"/>
-    <col min="20" max="20" width="7.08984375" customWidth="1"/>
+    <col min="1" max="1" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="31" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="7.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -529,46 +517,40 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>62</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>63</v>
+        <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="T1" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>7724</v>
       </c>
@@ -590,42 +572,38 @@
       <c r="G2" s="1">
         <v>6029930210</v>
       </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1" t="s">
-        <v>64</v>
+      <c r="H2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0.35416666666666669</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>21</v>
       </c>
       <c r="K2" s="2">
-        <v>0.35416666666666669</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M2" s="2">
         <v>0.53789351851851852</v>
       </c>
+      <c r="L2" s="1">
+        <v>2076</v>
+      </c>
+      <c r="M2" s="1">
+        <v>2098</v>
+      </c>
       <c r="N2" s="1">
-        <v>2076</v>
-      </c>
-      <c r="O2" s="1">
-        <v>2098</v>
-      </c>
-      <c r="P2" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S2" s="1">
-        <v>0</v>
-      </c>
-      <c r="T2" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>0</v>
+      </c>
+      <c r="R2" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>7724</v>
       </c>
@@ -647,42 +625,38 @@
       <c r="G3" s="1">
         <v>6029930211</v>
       </c>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1" t="s">
-        <v>65</v>
+      <c r="H3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="2">
+        <v>0.53789351851851852</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>21</v>
       </c>
       <c r="K3" s="2">
-        <v>0.53789351851851852</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M3" s="2">
         <v>0.72162037037037041</v>
       </c>
+      <c r="L3" s="1">
+        <v>2076</v>
+      </c>
+      <c r="M3" s="1">
+        <v>0</v>
+      </c>
       <c r="N3" s="1">
-        <v>2076</v>
-      </c>
-      <c r="O3" s="1">
-        <v>0</v>
-      </c>
-      <c r="P3" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S3" s="1">
-        <v>0</v>
-      </c>
-      <c r="T3" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>0</v>
+      </c>
+      <c r="R3" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>7724</v>
       </c>
@@ -704,40 +678,38 @@
       <c r="G4" s="1">
         <v>6029930212</v>
       </c>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
+      <c r="H4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0.72162037037037041</v>
+      </c>
       <c r="J4" s="1" t="s">
         <v>21</v>
       </c>
       <c r="K4" s="2">
-        <v>0.72162037037037041</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M4" s="2">
         <v>0.90534722222222219</v>
       </c>
+      <c r="L4" s="1">
+        <v>2076</v>
+      </c>
+      <c r="M4" s="1">
+        <v>0</v>
+      </c>
       <c r="N4" s="1">
-        <v>2076</v>
-      </c>
-      <c r="O4" s="1">
-        <v>0</v>
-      </c>
-      <c r="P4" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S4" s="1">
-        <v>0</v>
-      </c>
-      <c r="T4" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>0</v>
+      </c>
+      <c r="R4" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>7724</v>
       </c>
@@ -759,40 +731,38 @@
       <c r="G5" s="1">
         <v>6029930213</v>
       </c>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
+      <c r="H5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0.90534722222222219</v>
+      </c>
       <c r="J5" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K5" s="2">
-        <v>0.90534722222222219</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M5" s="2">
         <v>0.4224074074074074</v>
       </c>
+      <c r="L5" s="1">
+        <v>2076</v>
+      </c>
+      <c r="M5" s="1">
+        <v>0</v>
+      </c>
       <c r="N5" s="1">
-        <v>2076</v>
-      </c>
-      <c r="O5" s="1">
-        <v>0</v>
-      </c>
-      <c r="P5" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S5" s="1">
-        <v>0</v>
-      </c>
-      <c r="T5" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>0</v>
+      </c>
+      <c r="R5" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>7724</v>
       </c>
@@ -814,40 +784,38 @@
       <c r="G6" s="1">
         <v>6030930210</v>
       </c>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
+      <c r="H6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" s="2">
+        <v>0.4224074074074074</v>
+      </c>
       <c r="J6" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K6" s="2">
-        <v>0.4224074074074074</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M6" s="2">
         <v>0.60613425925925923</v>
       </c>
+      <c r="L6" s="1">
+        <v>2076</v>
+      </c>
+      <c r="M6" s="1">
+        <v>0</v>
+      </c>
       <c r="N6" s="1">
-        <v>2076</v>
-      </c>
-      <c r="O6" s="1">
-        <v>0</v>
-      </c>
-      <c r="P6" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S6" s="1">
-        <v>0</v>
-      </c>
-      <c r="T6" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>0</v>
+      </c>
+      <c r="R6" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>7724</v>
       </c>
@@ -869,40 +837,38 @@
       <c r="G7" s="1">
         <v>6030930211</v>
       </c>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
+      <c r="H7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0.60613425925925923</v>
+      </c>
       <c r="J7" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K7" s="2">
-        <v>0.60613425925925923</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M7" s="2">
         <v>0.78986111111111112</v>
       </c>
+      <c r="L7" s="1">
+        <v>2076</v>
+      </c>
+      <c r="M7" s="1">
+        <v>0</v>
+      </c>
       <c r="N7" s="1">
-        <v>2076</v>
-      </c>
-      <c r="O7" s="1">
-        <v>0</v>
-      </c>
-      <c r="P7" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S7" s="1">
-        <v>0</v>
-      </c>
-      <c r="T7" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q7" s="1">
+        <v>0</v>
+      </c>
+      <c r="R7" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7724</v>
       </c>
@@ -924,40 +890,38 @@
       <c r="G8" s="1">
         <v>6029930224</v>
       </c>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
+      <c r="H8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" s="2">
+        <v>0.33334490740740741</v>
+      </c>
       <c r="J8" s="1" t="s">
         <v>21</v>
       </c>
       <c r="K8" s="2">
-        <v>0.33334490740740741</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M8" s="2">
         <v>0.62872685185185184</v>
       </c>
+      <c r="L8" s="1">
+        <v>795</v>
+      </c>
+      <c r="M8" s="1">
+        <v>720</v>
+      </c>
       <c r="N8" s="1">
-        <v>795</v>
-      </c>
-      <c r="O8" s="1">
-        <v>720</v>
-      </c>
-      <c r="P8" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S8" s="1">
-        <v>0</v>
-      </c>
-      <c r="T8" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q8" s="1">
+        <v>0</v>
+      </c>
+      <c r="R8" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>7724</v>
       </c>
@@ -979,40 +943,38 @@
       <c r="G9" s="1">
         <v>6029930222</v>
       </c>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
+      <c r="H9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I9" s="2">
+        <v>0.62873842592592588</v>
+      </c>
       <c r="J9" s="1" t="s">
         <v>21</v>
       </c>
       <c r="K9" s="2">
-        <v>0.62873842592592588</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M9" s="2">
         <v>0.92412037037037043</v>
       </c>
+      <c r="L9" s="1">
+        <v>795</v>
+      </c>
+      <c r="M9" s="1">
+        <v>0</v>
+      </c>
       <c r="N9" s="1">
-        <v>795</v>
-      </c>
-      <c r="O9" s="1">
-        <v>0</v>
-      </c>
-      <c r="P9" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S9" s="1">
-        <v>0</v>
-      </c>
-      <c r="T9" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q9" s="1">
+        <v>0</v>
+      </c>
+      <c r="R9" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>7724</v>
       </c>
@@ -1034,40 +996,38 @@
       <c r="G10" s="1">
         <v>6029930242</v>
       </c>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
+      <c r="H10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I10" s="2">
+        <v>0.37501157407407409</v>
+      </c>
       <c r="J10" s="1" t="s">
         <v>21</v>
       </c>
       <c r="K10" s="2">
-        <v>0.37501157407407409</v>
-      </c>
-      <c r="L10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M10" s="2">
         <v>0.6189930555555555</v>
       </c>
+      <c r="L10" s="1">
+        <v>1660</v>
+      </c>
+      <c r="M10" s="1">
+        <v>1440</v>
+      </c>
       <c r="N10" s="1">
-        <v>1660</v>
-      </c>
-      <c r="O10" s="1">
-        <v>1440</v>
-      </c>
-      <c r="P10" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S10" s="1">
-        <v>0</v>
-      </c>
-      <c r="T10" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q10" s="1">
+        <v>0</v>
+      </c>
+      <c r="R10" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>7724</v>
       </c>
@@ -1089,40 +1049,38 @@
       <c r="G11" s="1">
         <v>6029930243</v>
       </c>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
+      <c r="H11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" s="2">
+        <v>0.61900462962962965</v>
+      </c>
       <c r="J11" s="1" t="s">
         <v>21</v>
       </c>
       <c r="K11" s="2">
-        <v>0.61900462962962965</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M11" s="2">
         <v>0.72574074074074069</v>
       </c>
+      <c r="L11" s="1">
+        <v>830</v>
+      </c>
+      <c r="M11" s="1">
+        <v>0</v>
+      </c>
       <c r="N11" s="1">
-        <v>830</v>
-      </c>
-      <c r="O11" s="1">
-        <v>0</v>
-      </c>
-      <c r="P11" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S11" s="1">
-        <v>0</v>
-      </c>
-      <c r="T11" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>0</v>
+      </c>
+      <c r="R11" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>7724</v>
       </c>
@@ -1144,43 +1102,41 @@
       <c r="G12" s="1">
         <v>6029930244</v>
       </c>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
+      <c r="H12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0.72574074074074069</v>
+      </c>
       <c r="J12" s="1" t="s">
         <v>21</v>
       </c>
       <c r="K12" s="2">
-        <v>0.72574074074074069</v>
-      </c>
-      <c r="L12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M12" s="2">
         <v>0.83253472222222225</v>
       </c>
+      <c r="L12" s="1">
+        <v>1038</v>
+      </c>
+      <c r="M12" s="1">
+        <v>0</v>
+      </c>
       <c r="N12" s="1">
-        <v>1038</v>
-      </c>
-      <c r="O12" s="1">
-        <v>0</v>
-      </c>
-      <c r="P12" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="R12" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="P12" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="S12" s="1">
-        <v>0</v>
-      </c>
-      <c r="T12" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q12" s="1">
+        <v>0</v>
+      </c>
+      <c r="R12" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>7724</v>
       </c>
@@ -1202,40 +1158,38 @@
       <c r="G13" s="1">
         <v>6029930245</v>
       </c>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
+      <c r="H13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I13" s="2">
+        <v>0.83253472222222225</v>
+      </c>
       <c r="J13" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K13" s="2">
-        <v>0.83253472222222225</v>
-      </c>
-      <c r="L13" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M13" s="2">
         <v>0.37945601851851851</v>
       </c>
+      <c r="L13" s="1">
+        <v>2076</v>
+      </c>
+      <c r="M13" s="1">
+        <v>0</v>
+      </c>
       <c r="N13" s="1">
-        <v>2076</v>
-      </c>
-      <c r="O13" s="1">
-        <v>0</v>
-      </c>
-      <c r="P13" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S13" s="1">
-        <v>0</v>
-      </c>
-      <c r="T13" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q13" s="1">
+        <v>0</v>
+      </c>
+      <c r="R13" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>7724</v>
       </c>
@@ -1257,40 +1211,38 @@
       <c r="G14" s="1">
         <v>6030930240</v>
       </c>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
+      <c r="H14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0.37945601851851851</v>
+      </c>
       <c r="J14" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K14" s="2">
-        <v>0.37945601851851851</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M14" s="2">
         <v>0.59304398148148152</v>
       </c>
+      <c r="L14" s="1">
+        <v>2076</v>
+      </c>
+      <c r="M14" s="1">
+        <v>0</v>
+      </c>
       <c r="N14" s="1">
-        <v>2076</v>
-      </c>
-      <c r="O14" s="1">
-        <v>0</v>
-      </c>
-      <c r="P14" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S14" s="1">
-        <v>0</v>
-      </c>
-      <c r="T14" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q14" s="1">
+        <v>0</v>
+      </c>
+      <c r="R14" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>7724</v>
       </c>
@@ -1312,40 +1264,38 @@
       <c r="G15" s="1">
         <v>6030930245</v>
       </c>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
+      <c r="H15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I15" s="2">
+        <v>0.59304398148148152</v>
+      </c>
       <c r="J15" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K15" s="2">
-        <v>0.59304398148148152</v>
-      </c>
-      <c r="L15" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M15" s="2">
         <v>0.80652777777777773</v>
       </c>
+      <c r="L15" s="1">
+        <v>2076</v>
+      </c>
+      <c r="M15" s="1">
+        <v>0</v>
+      </c>
       <c r="N15" s="1">
-        <v>2076</v>
-      </c>
-      <c r="O15" s="1">
-        <v>0</v>
-      </c>
-      <c r="P15" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S15" s="1">
-        <v>0</v>
-      </c>
-      <c r="T15" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q15" s="1">
+        <v>0</v>
+      </c>
+      <c r="R15" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>7724</v>
       </c>
@@ -1367,40 +1317,38 @@
       <c r="G16" s="1">
         <v>6029930268</v>
       </c>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
+      <c r="H16" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I16" s="2">
+        <v>0.50123842592592593</v>
+      </c>
       <c r="J16" s="1" t="s">
         <v>21</v>
       </c>
       <c r="K16" s="2">
-        <v>0.50123842592592593</v>
-      </c>
-      <c r="L16" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M16" s="2">
         <v>0.59559027777777773</v>
       </c>
+      <c r="L16" s="1">
+        <v>575</v>
+      </c>
+      <c r="M16" s="1">
+        <v>588</v>
+      </c>
       <c r="N16" s="1">
-        <v>575</v>
-      </c>
-      <c r="O16" s="1">
-        <v>588</v>
-      </c>
-      <c r="P16" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S16" s="1">
-        <v>0</v>
-      </c>
-      <c r="T16" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q16" s="1">
+        <v>0</v>
+      </c>
+      <c r="R16" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>7724</v>
       </c>
@@ -1422,40 +1370,38 @@
       <c r="G17" s="1">
         <v>6029930269</v>
       </c>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
+      <c r="H17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I17" s="2">
+        <v>0.59560185185185188</v>
+      </c>
       <c r="J17" s="1" t="s">
         <v>21</v>
       </c>
       <c r="K17" s="2">
-        <v>0.59560185185185188</v>
-      </c>
-      <c r="L17" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M17" s="2">
         <v>0.68995370370370368</v>
       </c>
+      <c r="L17" s="1">
+        <v>575</v>
+      </c>
+      <c r="M17" s="1">
+        <v>0</v>
+      </c>
       <c r="N17" s="1">
-        <v>575</v>
-      </c>
-      <c r="O17" s="1">
-        <v>0</v>
-      </c>
-      <c r="P17" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S17" s="1">
-        <v>0</v>
-      </c>
-      <c r="T17" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O17" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>0</v>
+      </c>
+      <c r="R17" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>7724</v>
       </c>
@@ -1477,40 +1423,38 @@
       <c r="G18" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
+      <c r="H18" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I18" s="2">
+        <v>0.68996527777777783</v>
+      </c>
       <c r="J18" s="1" t="s">
         <v>21</v>
       </c>
       <c r="K18" s="2">
-        <v>0.68996527777777783</v>
-      </c>
-      <c r="L18" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M18" s="2">
         <v>0.78431712962962963</v>
       </c>
+      <c r="L18" s="1">
+        <v>575</v>
+      </c>
+      <c r="M18" s="1">
+        <v>0</v>
+      </c>
       <c r="N18" s="1">
-        <v>575</v>
-      </c>
-      <c r="O18" s="1">
-        <v>0</v>
-      </c>
-      <c r="P18" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S18" s="1">
-        <v>0</v>
-      </c>
-      <c r="T18" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q18" s="1">
+        <v>0</v>
+      </c>
+      <c r="R18" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>7724</v>
       </c>
@@ -1532,43 +1476,41 @@
       <c r="G19" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
+      <c r="H19" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I19" s="2">
+        <v>0.78432870370370367</v>
+      </c>
       <c r="J19" s="1" t="s">
         <v>21</v>
       </c>
       <c r="K19" s="2">
-        <v>0.78432870370370367</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M19" s="2">
         <v>0.83026620370370374</v>
       </c>
+      <c r="L19" s="1">
+        <v>280</v>
+      </c>
+      <c r="M19" s="1">
+        <v>0</v>
+      </c>
       <c r="N19" s="1">
-        <v>280</v>
-      </c>
-      <c r="O19" s="1">
-        <v>0</v>
-      </c>
-      <c r="P19" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="R19" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="P19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="S19" s="1">
-        <v>0</v>
-      </c>
-      <c r="T19" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q19" s="1">
+        <v>0</v>
+      </c>
+      <c r="R19" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>7724</v>
       </c>
@@ -1590,43 +1532,41 @@
       <c r="G20" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
+      <c r="H20" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I20" s="2">
+        <v>0.83027777777777778</v>
+      </c>
       <c r="J20" s="1" t="s">
         <v>21</v>
       </c>
       <c r="K20" s="2">
-        <v>0.83027777777777778</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M20" s="2">
         <v>0.94701388888888893</v>
       </c>
+      <c r="L20" s="1">
+        <v>830</v>
+      </c>
+      <c r="M20" s="1">
+        <v>0</v>
+      </c>
       <c r="N20" s="1">
-        <v>830</v>
-      </c>
-      <c r="O20" s="1">
-        <v>0</v>
-      </c>
-      <c r="P20" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="R20" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="O20" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="P20" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="S20" s="1">
-        <v>0</v>
-      </c>
-      <c r="T20" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q20" s="1">
+        <v>0</v>
+      </c>
+      <c r="R20" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>7724</v>
       </c>
@@ -1648,43 +1588,41 @@
       <c r="G21" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
+      <c r="H21" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I21" s="2">
+        <v>0.94701388888888893</v>
+      </c>
       <c r="J21" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K21" s="2">
-        <v>0.94701388888888893</v>
-      </c>
-      <c r="L21" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M21" s="2">
         <v>0.12887731481481482</v>
       </c>
+      <c r="L21" s="1">
+        <v>1293</v>
+      </c>
+      <c r="M21" s="1">
+        <v>0</v>
+      </c>
       <c r="N21" s="1">
-        <v>1293</v>
-      </c>
-      <c r="O21" s="1">
-        <v>0</v>
-      </c>
-      <c r="P21" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="R21" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="P21" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="S21" s="1">
-        <v>0</v>
-      </c>
-      <c r="T21" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q21" s="1">
+        <v>0</v>
+      </c>
+      <c r="R21" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>7724</v>
       </c>
@@ -1706,43 +1644,41 @@
       <c r="G22" s="1">
         <v>6030930263</v>
       </c>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
+      <c r="H22" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I22" s="2">
+        <v>0.12887731481481482</v>
+      </c>
       <c r="J22" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K22" s="2">
-        <v>0.12887731481481482</v>
-      </c>
-      <c r="L22" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M22" s="2">
         <v>0.20061342592592593</v>
       </c>
+      <c r="L22" s="1">
+        <v>680</v>
+      </c>
+      <c r="M22" s="1">
+        <v>0</v>
+      </c>
       <c r="N22" s="1">
-        <v>680</v>
-      </c>
-      <c r="O22" s="1">
-        <v>0</v>
-      </c>
-      <c r="P22" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="R22" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="O22" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="P22" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="S22" s="1">
-        <v>0</v>
-      </c>
-      <c r="T22" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q22" s="1">
+        <v>0</v>
+      </c>
+      <c r="R22" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>7724</v>
       </c>
@@ -1764,40 +1700,38 @@
       <c r="G23" s="1">
         <v>6030930263</v>
       </c>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
+      <c r="H23" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I23" s="2">
+        <v>0.20061342592592593</v>
+      </c>
       <c r="J23" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K23" s="2">
-        <v>0.20061342592592593</v>
-      </c>
-      <c r="L23" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M23" s="2">
         <v>0.32086805555555553</v>
       </c>
+      <c r="L23" s="1">
+        <v>1140</v>
+      </c>
+      <c r="M23" s="1">
+        <v>0</v>
+      </c>
       <c r="N23" s="1">
-        <v>1140</v>
-      </c>
-      <c r="O23" s="1">
-        <v>0</v>
-      </c>
-      <c r="P23" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S23" s="1">
-        <v>0</v>
-      </c>
-      <c r="T23" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O23" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q23" s="1">
+        <v>0</v>
+      </c>
+      <c r="R23" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>7724</v>
       </c>
@@ -1819,40 +1753,38 @@
       <c r="G24" s="1">
         <v>6030930267</v>
       </c>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
+      <c r="H24" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I24" s="2">
+        <v>0.32086805555555553</v>
+      </c>
       <c r="J24" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K24" s="2">
-        <v>0.32086805555555553</v>
-      </c>
-      <c r="L24" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M24" s="2">
         <v>0.38099537037037035</v>
       </c>
+      <c r="L24" s="1">
+        <v>570</v>
+      </c>
+      <c r="M24" s="1">
+        <v>0</v>
+      </c>
       <c r="N24" s="1">
-        <v>570</v>
-      </c>
-      <c r="O24" s="1">
-        <v>0</v>
-      </c>
-      <c r="P24" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S24" s="1">
-        <v>0</v>
-      </c>
-      <c r="T24" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q24" s="1">
+        <v>0</v>
+      </c>
+      <c r="R24" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>7724</v>
       </c>
@@ -1874,40 +1806,38 @@
       <c r="G25" s="1">
         <v>6030930268</v>
       </c>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
+      <c r="H25" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I25" s="2">
+        <v>0.38099537037037035</v>
+      </c>
       <c r="J25" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K25" s="2">
-        <v>0.38099537037037035</v>
-      </c>
-      <c r="L25" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M25" s="2">
         <v>0.44112268518518516</v>
       </c>
+      <c r="L25" s="1">
+        <v>570</v>
+      </c>
+      <c r="M25" s="1">
+        <v>0</v>
+      </c>
       <c r="N25" s="1">
-        <v>570</v>
-      </c>
-      <c r="O25" s="1">
-        <v>0</v>
-      </c>
-      <c r="P25" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S25" s="1">
-        <v>0</v>
-      </c>
-      <c r="T25" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O25" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q25" s="1">
+        <v>0</v>
+      </c>
+      <c r="R25" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>7724</v>
       </c>
@@ -1929,43 +1859,41 @@
       <c r="G26" s="1">
         <v>6030930269</v>
       </c>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
+      <c r="H26" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I26" s="2">
+        <v>0.44112268518518516</v>
+      </c>
       <c r="J26" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K26" s="2">
-        <v>0.44112268518518516</v>
-      </c>
-      <c r="L26" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M26" s="2">
         <v>0.45373842592592595</v>
       </c>
+      <c r="L26" s="1">
+        <v>131</v>
+      </c>
+      <c r="M26" s="1">
+        <v>0</v>
+      </c>
       <c r="N26" s="1">
-        <v>131</v>
-      </c>
-      <c r="O26" s="1">
-        <v>0</v>
-      </c>
-      <c r="P26" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="R26" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="O26" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="P26" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="S26" s="1">
-        <v>0</v>
-      </c>
-      <c r="T26" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q26" s="1">
+        <v>0</v>
+      </c>
+      <c r="R26" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>7724</v>
       </c>
@@ -1987,43 +1915,41 @@
       <c r="G27" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="H27" s="1"/>
-      <c r="I27" s="1"/>
+      <c r="H27" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I27" s="2">
+        <v>0.45373842592592595</v>
+      </c>
       <c r="J27" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K27" s="2">
-        <v>0.45373842592592595</v>
-      </c>
-      <c r="L27" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M27" s="2">
         <v>0.62759259259259259</v>
       </c>
+      <c r="L27" s="1">
+        <v>1235</v>
+      </c>
+      <c r="M27" s="1">
+        <v>0</v>
+      </c>
       <c r="N27" s="1">
-        <v>1235</v>
-      </c>
-      <c r="O27" s="1">
-        <v>0</v>
-      </c>
-      <c r="P27" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="R27" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="O27" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="P27" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="S27" s="1">
-        <v>0</v>
-      </c>
-      <c r="T27" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q27" s="1">
+        <v>0</v>
+      </c>
+      <c r="R27" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>7724</v>
       </c>
@@ -2045,40 +1971,38 @@
       <c r="G28" s="1">
         <v>6030930268</v>
       </c>
-      <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
+      <c r="H28" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I28" s="2">
+        <v>0.62759259259259259</v>
+      </c>
       <c r="J28" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K28" s="2">
-        <v>0.62759259259259259</v>
-      </c>
-      <c r="L28" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M28" s="2">
         <v>0.6878009259259259</v>
       </c>
+      <c r="L28" s="1">
+        <v>742</v>
+      </c>
+      <c r="M28" s="1">
+        <v>0</v>
+      </c>
       <c r="N28" s="1">
-        <v>742</v>
-      </c>
-      <c r="O28" s="1">
-        <v>0</v>
-      </c>
-      <c r="P28" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S28" s="1">
-        <v>0</v>
-      </c>
-      <c r="T28" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O28" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q28" s="1">
+        <v>0</v>
+      </c>
+      <c r="R28" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>7724</v>
       </c>
@@ -2100,40 +2024,38 @@
       <c r="G29" s="1">
         <v>6030930269</v>
       </c>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
+      <c r="H29" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I29" s="2">
+        <v>0.6878009259259259</v>
+      </c>
       <c r="J29" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K29" s="2">
-        <v>0.6878009259259259</v>
-      </c>
-      <c r="L29" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M29" s="2">
         <v>0.80821759259259263</v>
       </c>
+      <c r="L29" s="1">
+        <v>1484</v>
+      </c>
+      <c r="M29" s="1">
+        <v>0</v>
+      </c>
       <c r="N29" s="1">
-        <v>1484</v>
-      </c>
-      <c r="O29" s="1">
-        <v>0</v>
-      </c>
-      <c r="P29" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q29" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S29" s="1">
-        <v>0</v>
-      </c>
-      <c r="T29" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O29" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q29" s="1">
+        <v>0</v>
+      </c>
+      <c r="R29" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>7724</v>
       </c>
@@ -2155,40 +2077,38 @@
       <c r="G30" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
+      <c r="H30" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I30" s="2">
+        <v>0.80821759259259263</v>
+      </c>
       <c r="J30" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K30" s="2">
-        <v>0.80821759259259263</v>
-      </c>
-      <c r="L30" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M30" s="2">
         <v>0.86842592592592593</v>
       </c>
+      <c r="L30" s="1">
+        <v>742</v>
+      </c>
+      <c r="M30" s="1">
+        <v>0</v>
+      </c>
       <c r="N30" s="1">
-        <v>742</v>
-      </c>
-      <c r="O30" s="1">
-        <v>0</v>
-      </c>
-      <c r="P30" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S30" s="1">
-        <v>0</v>
-      </c>
-      <c r="T30" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O30" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q30" s="1">
+        <v>0</v>
+      </c>
+      <c r="R30" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>7724</v>
       </c>
@@ -2210,40 +2130,38 @@
       <c r="G31" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
+      <c r="H31" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I31" s="2">
+        <v>0.86842592592592593</v>
+      </c>
       <c r="J31" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K31" s="2">
-        <v>0.86842592592592593</v>
-      </c>
-      <c r="L31" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M31" s="2">
         <v>0.92863425925925924</v>
       </c>
+      <c r="L31" s="1">
+        <v>742</v>
+      </c>
+      <c r="M31" s="1">
+        <v>0</v>
+      </c>
       <c r="N31" s="1">
-        <v>742</v>
-      </c>
-      <c r="O31" s="1">
-        <v>0</v>
-      </c>
-      <c r="P31" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q31" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S31" s="1">
-        <v>0</v>
-      </c>
-      <c r="T31" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O31" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q31" s="1">
+        <v>0</v>
+      </c>
+      <c r="R31" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>7724</v>
       </c>
@@ -2265,40 +2183,38 @@
       <c r="G32" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
+      <c r="H32" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I32" s="2">
+        <v>0.92863425925925924</v>
+      </c>
       <c r="J32" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K32" s="2">
-        <v>0.92863425925925924</v>
-      </c>
-      <c r="L32" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M32" s="2">
         <v>0.97940972222222222</v>
       </c>
+      <c r="L32" s="1">
+        <v>722</v>
+      </c>
+      <c r="M32" s="1">
+        <v>0</v>
+      </c>
       <c r="N32" s="1">
-        <v>722</v>
-      </c>
-      <c r="O32" s="1">
-        <v>0</v>
-      </c>
-      <c r="P32" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q32" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S32" s="1">
-        <v>0</v>
-      </c>
-      <c r="T32" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O32" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q32" s="1">
+        <v>0</v>
+      </c>
+      <c r="R32" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>7724</v>
       </c>
@@ -2320,40 +2236,38 @@
       <c r="G33" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="H33" s="1"/>
-      <c r="I33" s="1"/>
+      <c r="H33" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I33" s="2">
+        <v>0.97940972222222222</v>
+      </c>
       <c r="J33" s="1" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="K33" s="2">
-        <v>0.97940972222222222</v>
-      </c>
-      <c r="L33" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="M33" s="2">
         <v>3.0185185185185186E-2</v>
       </c>
+      <c r="L33" s="1">
+        <v>722</v>
+      </c>
+      <c r="M33" s="1">
+        <v>0</v>
+      </c>
       <c r="N33" s="1">
-        <v>722</v>
-      </c>
-      <c r="O33" s="1">
-        <v>0</v>
-      </c>
-      <c r="P33" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q33" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S33" s="1">
-        <v>0</v>
-      </c>
-      <c r="T33" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O33" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q33" s="1">
+        <v>0</v>
+      </c>
+      <c r="R33" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>7724</v>
       </c>
@@ -2375,40 +2289,38 @@
       <c r="G34" s="1">
         <v>6029930280</v>
       </c>
-      <c r="H34" s="1"/>
-      <c r="I34" s="1"/>
+      <c r="H34" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I34" s="2">
+        <v>0.37314814814814817</v>
+      </c>
       <c r="J34" s="1" t="s">
         <v>21</v>
       </c>
       <c r="K34" s="2">
-        <v>0.37314814814814817</v>
-      </c>
-      <c r="L34" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M34" s="2">
         <v>0.57337962962962963</v>
       </c>
+      <c r="L34" s="1">
+        <v>300</v>
+      </c>
+      <c r="M34" s="1">
+        <v>0</v>
+      </c>
       <c r="N34" s="1">
-        <v>300</v>
-      </c>
-      <c r="O34" s="1">
-        <v>0</v>
-      </c>
-      <c r="P34" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q34" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S34" s="1">
-        <v>0</v>
-      </c>
-      <c r="T34" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O34" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q34" s="1">
+        <v>0</v>
+      </c>
+      <c r="R34" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>7724</v>
       </c>
@@ -2430,40 +2342,38 @@
       <c r="G35" s="1">
         <v>6029930280</v>
       </c>
-      <c r="H35" s="1"/>
-      <c r="I35" s="1"/>
+      <c r="H35" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I35" s="2">
+        <v>0.57337962962962963</v>
+      </c>
       <c r="J35" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K35" s="2">
-        <v>0.57337962962962963</v>
-      </c>
-      <c r="L35" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M35" s="2">
         <v>0.40913194444444445</v>
       </c>
+      <c r="L35" s="1">
+        <v>200</v>
+      </c>
+      <c r="M35" s="1">
+        <v>0</v>
+      </c>
       <c r="N35" s="1">
-        <v>200</v>
-      </c>
-      <c r="O35" s="1">
-        <v>0</v>
-      </c>
-      <c r="P35" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q35" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S35" s="1">
-        <v>0</v>
-      </c>
-      <c r="T35" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="O35" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q35" s="1">
+        <v>0</v>
+      </c>
+      <c r="R35" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>7724</v>
       </c>
@@ -2485,36 +2395,34 @@
       <c r="G36" s="1">
         <v>6030930280</v>
       </c>
-      <c r="H36" s="1"/>
-      <c r="I36" s="1"/>
+      <c r="H36" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I36" s="2">
+        <v>0.40913194444444445</v>
+      </c>
       <c r="J36" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K36" s="2">
-        <v>0.40913194444444445</v>
-      </c>
-      <c r="L36" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M36" s="2">
         <v>0.50780092592592596</v>
       </c>
+      <c r="L36" s="1">
+        <v>300</v>
+      </c>
+      <c r="M36" s="1">
+        <v>0</v>
+      </c>
       <c r="N36" s="1">
-        <v>300</v>
-      </c>
-      <c r="O36" s="1">
-        <v>0</v>
-      </c>
-      <c r="P36" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q36" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S36" s="1">
-        <v>0</v>
-      </c>
-      <c r="T36" s="1">
+        <v>0</v>
+      </c>
+      <c r="O36" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q36" s="1">
+        <v>0</v>
+      </c>
+      <c r="R36" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>